<commit_message>
elhd.py anterior, revisar que al actualizarlo el consumo promedio subio en ves de bajar
</commit_message>
<xml_diff>
--- a/data/data_chuqui_3mb_onboard_fixed_validacion/elmo_data.xlsx
+++ b/data/data_chuqui_3mb_onboard_fixed_validacion/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\data_chuqui_3mb_onboard_fixed_validacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7AD0E2-F2FA-4B46-A171-DADC72910FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716CFD3A-6424-41DC-A740-4E67B5BE6D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batteries" sheetId="1" r:id="rId1"/>
@@ -3971,7 +3971,7 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -4070,10 +4070,10 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>2100</v>
+        <v>10000</v>
       </c>
       <c r="G3">
-        <v>2100</v>
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>